<commit_message>
chore: rebuild deliverables 2026-05-01
</commit_message>
<xml_diff>
--- a/data/public/bcn_transit_master.xlsx
+++ b/data/public/bcn_transit_master.xlsx
@@ -559,7 +559,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>5,016,052</t>
+          <t>5,189,019</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -569,22 +569,22 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>▲ 5.9% vs Apr 2025 (4,736,423 → 5,016,052)</t>
+          <t>▲ 9.6% vs Apr 2025 (4,736,423 → 5,189,019)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>▼ 7.2% vs Mar 2026 (5,403,169 → 5,016,052)</t>
+          <t>▼ 4.0% vs Mar 2026 (5,403,169 → 5,189,019)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>46.5% of Apr 2019 (10,779,665 baseline)</t>
+          <t>48.1% of Apr 2019 (10,779,665 baseline)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Large month-over-month swing (-7.2%) | Provisional — partial month, may be revised</t>
+          <t>Provisional — partial month, may be revised</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1365,7 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2009,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2515,7 +2515,7 @@
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="L60" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="L62" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="L64" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="L66" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="L67" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="L68" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="L70" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="L71" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -3987,7 +3987,7 @@
       </c>
       <c r="L73" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="L75" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="L77" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4217,7 +4217,7 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="L79" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4355,7 +4355,7 @@
       </c>
       <c r="L81" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="L83" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4539,7 +4539,7 @@
       </c>
       <c r="L85" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="L87" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4677,7 +4677,7 @@
       </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4723,7 +4723,7 @@
       </c>
       <c r="L89" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4769,7 +4769,7 @@
       </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="L91" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4861,7 +4861,7 @@
       </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
       </c>
       <c r="L93" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4953,7 +4953,7 @@
       </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="L95" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5045,7 +5045,7 @@
       </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="L97" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5137,7 +5137,7 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="L99" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="L101" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="L103" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5459,7 +5459,7 @@
       </c>
       <c r="L105" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5505,7 +5505,7 @@
       </c>
       <c r="L106" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="L107" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="L109" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5689,7 +5689,7 @@
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="L111" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5781,7 +5781,7 @@
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5827,7 +5827,7 @@
       </c>
       <c r="L113" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5873,7 +5873,7 @@
       </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="L115" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -5965,7 +5965,7 @@
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6011,7 +6011,7 @@
       </c>
       <c r="L117" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6103,7 @@
       </c>
       <c r="L119" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6149,7 @@
       </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6195,7 +6195,7 @@
       </c>
       <c r="L121" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6241,7 @@
       </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6287,7 +6287,7 @@
       </c>
       <c r="L123" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="L125" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="L127" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6517,7 +6517,7 @@
       </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6563,7 +6563,7 @@
       </c>
       <c r="L129" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6609,7 +6609,7 @@
       </c>
       <c r="L130" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6655,7 +6655,7 @@
       </c>
       <c r="L131" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="L132" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6747,7 +6747,7 @@
       </c>
       <c r="L133" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6793,7 +6793,7 @@
       </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6839,7 @@
       </c>
       <c r="L135" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="L136" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6931,7 +6931,7 @@
       </c>
       <c r="L137" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -6977,7 +6977,7 @@
       </c>
       <c r="L138" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="L139" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="L140" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -7115,7 +7115,7 @@
       </c>
       <c r="L141" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -7161,7 +7161,7 @@
       </c>
       <c r="L142" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -7207,7 +7207,7 @@
       </c>
       <c r="L143" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:45Z</t>
         </is>
       </c>
     </row>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="L144" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7299,7 +7299,7 @@
       </c>
       <c r="L145" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7391,7 +7391,7 @@
       </c>
       <c r="L147" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7437,7 +7437,7 @@
       </c>
       <c r="L148" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7483,7 +7483,7 @@
       </c>
       <c r="L149" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="L150" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7575,7 +7575,7 @@
       </c>
       <c r="L151" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="L152" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7667,7 +7667,7 @@
       </c>
       <c r="L153" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7713,7 +7713,7 @@
       </c>
       <c r="L154" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7759,7 +7759,7 @@
       </c>
       <c r="L155" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="L156" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
       </c>
       <c r="L157" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7897,7 +7897,7 @@
       </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7943,7 +7943,7 @@
       </c>
       <c r="L159" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -7989,7 +7989,7 @@
       </c>
       <c r="L160" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8035,7 +8035,7 @@
       </c>
       <c r="L161" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="L162" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8127,7 +8127,7 @@
       </c>
       <c r="L163" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8173,7 +8173,7 @@
       </c>
       <c r="L164" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
       </c>
       <c r="L165" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8265,7 +8265,7 @@
       </c>
       <c r="L166" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8311,7 +8311,7 @@
       </c>
       <c r="L167" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8357,7 +8357,7 @@
       </c>
       <c r="L168" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8403,7 +8403,7 @@
       </c>
       <c r="L169" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8449,7 +8449,7 @@
       </c>
       <c r="L170" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8495,7 +8495,7 @@
       </c>
       <c r="L171" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8541,7 +8541,7 @@
       </c>
       <c r="L172" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8587,7 +8587,7 @@
       </c>
       <c r="L173" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8633,7 +8633,7 @@
       </c>
       <c r="L174" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="L175" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8725,7 +8725,7 @@
       </c>
       <c r="L176" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8771,7 +8771,7 @@
       </c>
       <c r="L177" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="L178" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8863,7 +8863,7 @@
       </c>
       <c r="L179" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8909,7 +8909,7 @@
       </c>
       <c r="L180" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -8955,7 +8955,7 @@
       </c>
       <c r="L181" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9001,7 +9001,7 @@
       </c>
       <c r="L182" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9047,7 +9047,7 @@
       </c>
       <c r="L183" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9093,7 +9093,7 @@
       </c>
       <c r="L184" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9139,7 +9139,7 @@
       </c>
       <c r="L185" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9185,7 @@
       </c>
       <c r="L186" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9231,7 +9231,7 @@
       </c>
       <c r="L187" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9277,7 +9277,7 @@
       </c>
       <c r="L188" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9323,7 +9323,7 @@
       </c>
       <c r="L189" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="L190" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9415,7 +9415,7 @@
       </c>
       <c r="L191" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9461,7 +9461,7 @@
       </c>
       <c r="L192" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="L193" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9553,7 +9553,7 @@
       </c>
       <c r="L194" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9599,7 +9599,7 @@
       </c>
       <c r="L195" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9645,7 +9645,7 @@
       </c>
       <c r="L196" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9691,7 +9691,7 @@
       </c>
       <c r="L197" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9737,7 +9737,7 @@
       </c>
       <c r="L198" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="L199" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9829,7 +9829,7 @@
       </c>
       <c r="L200" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9875,7 +9875,7 @@
       </c>
       <c r="L201" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9921,7 +9921,7 @@
       </c>
       <c r="L202" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -9967,7 +9967,7 @@
       </c>
       <c r="L203" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10013,7 +10013,7 @@
       </c>
       <c r="L204" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10059,7 +10059,7 @@
       </c>
       <c r="L205" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10105,7 +10105,7 @@
       </c>
       <c r="L206" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10151,7 +10151,7 @@
       </c>
       <c r="L207" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10197,7 +10197,7 @@
       </c>
       <c r="L208" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:25:59Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10243,7 +10243,7 @@
       </c>
       <c r="L209" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10289,7 +10289,7 @@
       </c>
       <c r="L210" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10335,7 +10335,7 @@
       </c>
       <c r="L211" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10381,7 +10381,7 @@
       </c>
       <c r="L212" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10427,7 +10427,7 @@
       </c>
       <c r="L213" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10473,7 +10473,7 @@
       </c>
       <c r="L214" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10519,7 +10519,7 @@
       </c>
       <c r="L215" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="L216" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10611,7 +10611,7 @@
       </c>
       <c r="L217" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10657,7 +10657,7 @@
       </c>
       <c r="L218" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10703,7 +10703,7 @@
       </c>
       <c r="L219" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10749,7 +10749,7 @@
       </c>
       <c r="L220" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10795,7 +10795,7 @@
       </c>
       <c r="L221" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10841,7 +10841,7 @@
       </c>
       <c r="L222" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="L223" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10933,7 +10933,7 @@
       </c>
       <c r="L224" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -10979,7 +10979,7 @@
       </c>
       <c r="L225" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11025,7 +11025,7 @@
       </c>
       <c r="L226" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11071,7 +11071,7 @@
       </c>
       <c r="L227" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11117,7 +11117,7 @@
       </c>
       <c r="L228" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11163,7 +11163,7 @@
       </c>
       <c r="L229" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11209,7 +11209,7 @@
       </c>
       <c r="L230" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11255,7 +11255,7 @@
       </c>
       <c r="L231" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11301,7 +11301,7 @@
       </c>
       <c r="L232" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11347,7 +11347,7 @@
       </c>
       <c r="L233" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11393,7 +11393,7 @@
       </c>
       <c r="L234" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11439,7 +11439,7 @@
       </c>
       <c r="L235" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11485,7 +11485,7 @@
       </c>
       <c r="L236" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11531,7 +11531,7 @@
       </c>
       <c r="L237" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11577,7 +11577,7 @@
       </c>
       <c r="L238" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11623,7 +11623,7 @@
       </c>
       <c r="L239" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11669,7 +11669,7 @@
       </c>
       <c r="L240" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11715,7 +11715,7 @@
       </c>
       <c r="L241" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11761,7 +11761,7 @@
       </c>
       <c r="L242" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11807,7 +11807,7 @@
       </c>
       <c r="L243" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11853,7 +11853,7 @@
       </c>
       <c r="L244" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11899,7 +11899,7 @@
       </c>
       <c r="L245" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11945,7 +11945,7 @@
       </c>
       <c r="L246" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -11991,7 +11991,7 @@
       </c>
       <c r="L247" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12037,7 +12037,7 @@
       </c>
       <c r="L248" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12083,7 +12083,7 @@
       </c>
       <c r="L249" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12129,7 +12129,7 @@
       </c>
       <c r="L250" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12175,7 +12175,7 @@
       </c>
       <c r="L251" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12221,7 +12221,7 @@
       </c>
       <c r="L252" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12267,7 +12267,7 @@
       </c>
       <c r="L253" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12313,7 +12313,7 @@
       </c>
       <c r="L254" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12359,7 +12359,7 @@
       </c>
       <c r="L255" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12405,7 +12405,7 @@
       </c>
       <c r="L256" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12451,7 +12451,7 @@
       </c>
       <c r="L257" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12497,7 +12497,7 @@
       </c>
       <c r="L258" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12543,7 +12543,7 @@
       </c>
       <c r="L259" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12589,7 +12589,7 @@
       </c>
       <c r="L260" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12635,7 +12635,7 @@
       </c>
       <c r="L261" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12681,7 +12681,7 @@
       </c>
       <c r="L262" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12727,7 +12727,7 @@
       </c>
       <c r="L263" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12773,7 +12773,7 @@
       </c>
       <c r="L264" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12819,7 +12819,7 @@
       </c>
       <c r="L265" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12865,7 +12865,7 @@
       </c>
       <c r="L266" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12911,7 +12911,7 @@
       </c>
       <c r="L267" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -12957,7 +12957,7 @@
       </c>
       <c r="L268" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13003,7 +13003,7 @@
       </c>
       <c r="L269" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13049,7 +13049,7 @@
       </c>
       <c r="L270" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13095,7 +13095,7 @@
       </c>
       <c r="L271" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13141,7 +13141,7 @@
       </c>
       <c r="L272" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13187,7 +13187,7 @@
       </c>
       <c r="L273" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13233,7 +13233,7 @@
       </c>
       <c r="L274" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13279,7 +13279,7 @@
       </c>
       <c r="L275" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13325,7 +13325,7 @@
       </c>
       <c r="L276" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13371,7 +13371,7 @@
       </c>
       <c r="L277" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13425,7 @@
       </c>
       <c r="L278" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13479,7 +13479,7 @@
       </c>
       <c r="L279" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13533,7 +13533,7 @@
       </c>
       <c r="L280" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13587,7 +13587,7 @@
       </c>
       <c r="L281" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13641,7 +13641,7 @@
       </c>
       <c r="L282" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13695,7 +13695,7 @@
       </c>
       <c r="L283" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13749,7 +13749,7 @@
       </c>
       <c r="L284" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="L285" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13857,7 +13857,7 @@
       </c>
       <c r="L286" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13911,7 +13911,7 @@
       </c>
       <c r="L287" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -13965,7 +13965,7 @@
       </c>
       <c r="L288" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -14019,7 +14019,7 @@
       </c>
       <c r="L289" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -14073,7 +14073,7 @@
       </c>
       <c r="L290" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -14127,7 +14127,7 @@
       </c>
       <c r="L291" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -14171,7 +14171,7 @@
       </c>
       <c r="L292" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -14200,7 +14200,7 @@
         </is>
       </c>
       <c r="F293" s="4" t="n">
-        <v>5016052</v>
+        <v>5189019</v>
       </c>
       <c r="G293" s="4" t="inlineStr">
         <is>
@@ -14215,7 +14215,7 @@
       </c>
       <c r="L293" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01T05:26:00Z</t>
+          <t>2026-05-01T06:00:46Z</t>
         </is>
       </c>
     </row>
@@ -16002,7 +16002,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>5016052</v>
+        <v>5189019</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>5403169</v>
@@ -16956,17 +16956,17 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>5016052</v>
+        <v>5189019</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>4736423</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>279629</v>
+        <v>452596</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>+5.9%</t>
+          <t>+9.6%</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -26276,7 +26276,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Last updated: May 01, 2026 at 05:34 UTC</t>
+          <t>Last updated: May 01, 2026 at 06:00 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Muni recovery % uses SFMTA baseline in both Summary tab and Datawrapper CSVs
</commit_message>
<xml_diff>
--- a/data/public/bcn_transit_master.xlsx
+++ b/data/public/bcn_transit_master.xlsx
@@ -500,7 +500,7 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
     <col width="39" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -621,7 +621,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>109.9% of Mar 2019 (13,548,774 baseline)</t>
+          <t>84.4% of Mar 2019 (17,642,000 SFMTA baseline)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -50086,7 +50086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -50103,7 +50103,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Last updated: May 02, 2026 at 22:10 UTC</t>
+          <t>Last updated: May 02, 2026 at 22:20 UTC</t>
         </is>
       </c>
     </row>
@@ -50270,34 +50270,80 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
+          <t>sfmta.com</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Muni total boardings. Scraped automatically each weekday at 6 AM PT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
           <t>NTD Monthly</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>National Transit Database. ~2 month lag. Adjusted and finalized.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr"/>
-    </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>CONTACT</t>
-        </is>
-      </c>
+      <c r="A23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Andres Jimenez Larios | Bay City News</t>
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>NOTES</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Muni recovery %</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Uses SFMTA's own 2019 baseline — methodology matches SFMTA reporting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>BART recovery %</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Uses NTD 2019 same-month as baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>CONTACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Andres Jimenez Larios | Bay City News</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>GitHub: https://github.com/alariosjx/bcn-transit-tracker</t>
         </is>

</xml_diff>